<commit_message>
feat(F-NAR-019): ATOM-EMO.LEX.002-05 Victorino et le train en bois
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-EMO.LEX.002-05.xlsx
+++ b/stories/arbres/ATOM-EMO.LEX.002-05.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>chambre, puis salon</t>
+          <t>chambre, puis salon, coffre, train en bois, wagon, rail, lit, tapis, canapé, manteau, tasse</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Victorino ne trouve pas son train en bois. Il dit qu'il est triste. Il demande un câlin. Plus tard, Amir rentre chez lui. Victorino nomme encore la tristesse.</t>
+          <t>La poignée du coffre est tiède. Sur le couvercle, un éclat de coffre luit. Victorino veut le train en bois, maintenant, avec Amir. Le train n'est pas là. Sourire parti. Poitrine serrée. Yeux chauds. Papa s'accroupit. Victorino dit qu'il est triste. Il pleure. Il demande un câlin. Merci vécu. Deuxième ruse : Amir rentre chez lui, train toujours perdu. Il refuse de foncer. Un éclat de coffre tient sur le bois.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Une poussière danse dans la lumière. Le rayon arrive jusqu'au tapis. Un rail de bois attend sous le lit. L'horloge du couloir fait tic, tic. Un wagon rouge attend sur la chaise. Victorino, tu ranges les wagons ? Oui. Avec le train. Je plie la couverture. En ce moment, Victorino cherche. Il cherche le train en bois. Il regarde le lit. Pas là. Il regarde sous le lit. Pas là. Le tapis est doux sous les genoux. Papa, il n'est pas là. On cherche ensemble. Parce que le train n'est pas là. Victorino sent sa gorge serrée. Ses yeux deviennent chauds. Une larme tombe. Je suis triste. Tu es triste. C'est permis. Pleurer est permis. Victorino pleure un peu. Les larmes coulent. Elles sont chaudes. Je t'écoute, Victorino. Je veux un câlin. Viens. Un câlin. Papa ouvre les bras. Victorino se blottit. Le câlin est chaud. Le pull de papa sent le savon. Tu as dit : je suis triste. Bravo. Tu as demandé un câlin. Pleurer est permis, Victorino. Le câlin aide. Oui. Le câlin aide. Plus tard, au salon. Le canapé a une couverture rayée. Une tasse vide attend sur la table. Amir boutonne son manteau. Je rentre chez moi. Amir part, tout doucement. Victorino sent encore sa gorge. Je suis triste. Tu es triste. C'est permis. Pleurer est permis. Je veux un câlin. Viens. Un câlin. Maman le serre. Ses épaules se desserrent. Bravo. Tu as dit tes larmes. On peut demander un câlin. Le train, puis Amir. Le train, c'était pareil. La poussière danse encore.</t>
+          <t>La poignée du coffre est tiède, sous la fenêtre. Elle est chaude, papa. Tu la sens, la poignée ? Oui, papa. Amir est assis près du tapis, les genoux pliés. Ça sent le vernis. Tu le sens, Amir ? Oui, maman. La chambre sent le vernis, un peu. On fait le train, Amir ? Le train en bois, oui. Un wagon rouge attend sur la chaise, tout seul. Il manque le train. Un rail court un peu, près du lit. On va jusqu'au salon ? Oui, maintenant ! Vous partez tout de suite ? Oui, maman. Sur le couvercle, un éclat de coffre luit. Il brille, papa. Tu le vois, le petit point ? Oui, un grain clair. Il est sur le bois. Papa plie une couverture, près du lit. Je plie ça, d'accord ? Le train d'abord. En ce moment, Victorino cherche le train en bois. Je le veux, maintenant ! Tout de suite ? Oui, papa. Victorino fouille sous le lit, trop vite. Sa main sort, vide. Pas là. Sous le tapis ? Je regarde. Il soulève le tapis, trop vite. Le train n'est pas là. Papa, il n'est pas là. On cherche ensemble ? Oui. Amir ouvre le coffre, trop fort. Le couvercle claque contre le mur. Aïe, le bois. Il n'est pas dedans. Vous avez regardé au fond ? Vite, oui. Le sourire de Victorino disparaît. Dans sa poitrine, ça se serre. L'envie et la peur se heurtent. Ses épaules tombent un peu. J'ai mal au ventre. Ses yeux deviennent chauds. Une larme tombe sur le tapis. Je suis triste. Victorino pleure un peu, sans crier. Les larmes coulent sur ses joues. Tu as les yeux chauds, Victorino ? Oui, papa. Papa s'accroupit à la même hauteur. Tes mains sont chaudes, Victorino ? Un peu, maman. Je veux un câlin. Viens. Papa ouvre les bras. Victorino se blottit contre papa. Le câlin est chaud, près du cou. Ça sent le savon de papa. L'éclat de coffre tremble, puis tient.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Une poussière danse dans la lumière. Le rayon arrive jusqu'au tapis. Un rail de bois attend sous le lit. L'horloge du couloir fait tic, tic. Un wagon rouge attend sur la chaise. Victorino, tu ranges les wagons ? Oui. Avec le train. Je plie la couverture. En ce moment, Victorino cherche. Il cherche le train en bois. Il regarde le lit. Pas là. Il regarde sous le lit. Pas là. Le tapis est doux sous les genoux. Papa, il n'est pas là. On cherche ensemble. Parce que le train n'est pas là. Victorino sent sa gorge serrée. Ses yeux deviennent chauds. Une larme tombe. Je suis triste. Tu es triste. C'est permis. Pleurer est permis. Victorino pleure un peu. Les larmes coulent. Elles sont chaudes. Je t'écoute, Victorino. Je veux un câlin. Viens. Un câlin. Papa ouvre les bras. Victorino se blottit. Le câlin est chaud. Le pull de papa sent le savon. Tu as dit : je suis triste. Bravo. Tu as demandé un câlin. Pleurer est permis, Victorino. Le câlin aide. Oui. Le câlin aide. Plus tard, au salon. Le canapé a une couverture rayée. Une tasse vide attend sur la table. Amir boutonne son manteau. Je rentre chez moi. Amir part, tout doucement. Victorino sent encore sa gorge. Je suis triste. Tu es triste. C'est permis. Pleurer est permis. Je veux un câlin. Viens. Un câlin. Maman le serre. Ses épaules se desserrent. Bravo. Tu as dit tes larmes. On peut demander un câlin. Le train, puis Amir. Le train, c'était pareil. La poussière danse encore.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La poignée du coffre est tiède, sous la fenêtre. Elle est chaude, papa. Tu la sens, la poignée ? Oui, papa. Amir est assis près du tapis, les genoux pliés. Ça sent le vernis. Tu le sens, Amir ? Oui, maman. La chambre sent le vernis, un peu. On fait le train, Amir ? Le train en bois, oui. Un wagon rouge attend sur la chaise, tout seul. Il manque le train. Un rail court un peu, près du lit. On va jusqu'au salon ? Oui, maintenant ! Vous partez tout de suite ? Oui, maman. Sur le couvercle, un &lt;emphasis level="moderate"&gt;éclat de coffre&lt;/emphasis&gt; luit. Il brille, papa. Tu le vois, le petit point ? Oui, un grain clair. Il est sur le bois. Papa plie une couverture, près du lit. Je plie ça, d'accord ? Le train d'abord. En ce moment, Victorino cherche le train en bois. Je le veux, maintenant ! Tout de suite ? Oui, papa. Victorino fouille sous le lit, trop vite. Sa main sort, vide. Pas là. Sous le tapis ? Je regarde. Il soulève le tapis, trop vite. Le train n'est pas là. Papa, il n'est pas là. On cherche ensemble ? Oui. Amir ouvre le coffre, trop fort. Le couvercle claque contre le mur. Aïe, le bois. Il n'est pas dedans. Vous avez regardé au fond ? Vite, oui. Le sourire de Victorino disparaît. Dans sa poitrine, ça se serre. L'envie et la peur se heurtent. Ses épaules tombent un peu. J'ai mal au ventre. Ses yeux deviennent chauds. Une larme tombe sur le tapis. Je suis triste. Victorino pleure un peu, sans crier. Les larmes coulent sur ses joues. Tu as les yeux chauds, Victorino ? Oui, papa. Papa s'accroupit à la même hauteur. Tes mains sont chaudes, Victorino ? Un peu, maman. Je veux un câlin. Viens. Papa ouvre les bras. Victorino se blottit contre papa. Le câlin est chaud, près du cou. Ça sent le savon de papa. L'éclat de coffre tremble, puis tient.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Étienne cherche son train en bois dans la chambre. Le train n'est pas sous le lit. Étienne sent sa gorge serrée. Ses yeux deviennent chauds. Une larme tombe. Étienne dit : je suis &lt;emphasis&gt;triste&lt;/emphasis&gt;. Papa arrive près de lui. Papa dit : pleurer est permis. Étienne pleure un peu. Les larmes coulent. Puis Étienne dit : je veux un câlin. Papa ouvre les bras. Étienne se blottit. Le câlin est chaud. Parce que le train est perdu, Étienne est triste. Être triste, c'est permis. Plus tard, au salon, un camarade rentre chez lui. Étienne sent encore sa gorge. Il dit : je suis triste. Maman dit : pleurer est permis. Étienne demande un câlin. Maman le serre. Ses épaules se desserrent. Même leçon, autre moment. On nomme. On peut pleurer. On demande un câlin. [pause]</t>
+          <t>La poignée du coffre est tiède, sous la fenêtre. Elle est chaude, papa. Tu la sens, la poignée ? Oui, papa. Amir est assis près du tapis, les genoux pliés. Ça sent le vernis. Tu le sens, Amir ? Oui, maman. La chambre sent le vernis, un peu. On fait le train, Amir ? Le train en bois, oui. Un wagon rouge attend sur la chaise, tout seul. Il manque le train. Un rail court un peu, près du lit. On va jusqu'au salon ? Oui, maintenant ! Vous partez tout de suite ? Oui, maman. Sur le couvercle, un &lt;emphasis&gt;éclat de coffre&lt;/emphasis&gt; luit. Il brille, papa. Tu le vois, le petit point ? Oui, un grain clair. Il est sur le bois. Papa plie une couverture, près du lit. Je plie ça, d'accord ? Le train d'abord. En ce moment, Victorino cherche le train en bois. Je le veux, maintenant ! Tout de suite ? Oui, papa. Victorino fouille sous le lit, trop vite. Sa main sort, vide. Pas là. Sous le tapis ? Je regarde. Il soulève le tapis, trop vite. Le train n'est pas là. Papa, il n'est pas là. On cherche ensemble ? Oui. Amir ouvre le coffre, trop fort. Le couvercle claque contre le mur. Aïe, le bois. Il n'est pas dedans. Vous avez regardé au fond ? Vite, oui. Le sourire de Victorino disparaît. Dans sa poitrine, ça se serre. L'envie et la peur se heurtent. Ses épaules tombent un peu. J'ai mal au ventre. Ses yeux deviennent chauds. Une larme tombe sur le tapis. Je suis triste. Victorino pleure un peu, sans crier. Les larmes coulent sur ses joues. Tu as les yeux chauds, Victorino ? Oui, papa. Papa s'accroupit à la même hauteur. Tes mains sont chaudes, Victorino ? Un peu, maman. Je veux un câlin. Viens. Papa ouvre les bras. Victorino se blottit contre papa. Le câlin est chaud, près du cou. Ça sent le savon de papa. L'éclat de coffre tremble, puis tient. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,7 +1249,7 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
         <v>1.12</v>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>triste</t>
+          <t>éclat de coffre</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,64 +1321,86 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis tristesse; intensite=2; destinataire=enfant; sous_texte=il_veut_le_train_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Une poussière danse dans la lumière.
-narrateur|Le rayon arrive jusqu'au tapis.
-narrateur|Un rail de bois attend sous le lit.
-narrateur|L'horloge du couloir fait tic, tic.
-narrateur|Un wagon rouge attend sur la chaise.
-maman|Victorino, tu ranges les wagons ?
-enfant-m|Oui. Avec le train.
-papa|Je plie la couverture.
-narrateur|En ce moment, Victorino cherche.
-narrateur|Il cherche le train en bois.
-narrateur|Il regarde le lit. Pas là.
-narrateur|Il regarde sous le lit. Pas là.
-narrateur|Le tapis est doux sous les genoux.
+          <t>narrateur|La poignée du coffre est tiède, sous la fenêtre.
+enfant-m|Elle est chaude, papa.
+papa|Tu la sens, la poignée ?
+enfant-m|Oui, papa.
+narrateur|Amir est assis près du tapis, les genoux pliés.
+copain|Ça sent le vernis.
+maman|Tu le sens, Amir ?
+copain|Oui, maman.
+narrateur|La chambre sent le vernis, un peu.
+enfant-m|On fait le train, Amir ?
+copain|Le train en bois, oui.
+narrateur|Un wagon rouge attend sur la chaise, tout seul.
+enfant-m|Il manque le train.
+narrateur|Un rail court un peu, près du lit.
+copain|On va jusqu'au salon ?
+enfant-m|Oui, maintenant !
+maman|Vous partez tout de suite ?
+enfant-m|Oui, maman.
+narrateur|Sur le couvercle, un éclat de coffre luit.
+enfant-m|Il brille, papa.
+papa|Tu le vois, le petit point ?
+enfant-m|Oui, un grain clair.
+copain|Il est sur le bois.
+narrateur|Papa plie une couverture, près du lit.
+papa|Je plie ça, d'accord ?
+enfant-m|Le train d'abord.
+narrateur|En ce moment, Victorino cherche le train en bois.
+enfant-m|Je le veux, maintenant !
+papa|Tout de suite ?
+enfant-m|Oui, papa.
+narrateur|Victorino fouille sous le lit, trop vite.
+narrateur|Sa main sort, vide.
+enfant-m|Pas là.
+copain|Sous le tapis ?
+enfant-m|Je regarde.
+narrateur|Il soulève le tapis, trop vite.
+narrateur|Le train n'est pas là.
 enfant-m|Papa, il n'est pas là.
-papa|On cherche ensemble.
-narrateur|Parce que le train n'est pas là.
-narrateur|Victorino sent sa gorge serrée.
+papa|On cherche ensemble ?
+enfant-m|Oui.
+narrateur|Amir ouvre le coffre, trop fort.
+narrateur|Le couvercle claque contre le mur.
+copain|Aïe, le bois.
+enfant-m|Il n'est pas dedans.
+maman|Vous avez regardé au fond ?
+enfant-m|Vite, oui.
+narrateur|Le sourire de Victorino disparaît.
+narrateur|Dans sa poitrine, ça se serre.
+narrateur|L'envie et la peur se heurtent.
+narrateur|Ses épaules tombent un peu.
+enfant-m|J'ai mal au ventre.
 narrateur|Ses yeux deviennent chauds.
-narrateur|Une larme tombe.
+narrateur|Une larme tombe sur le tapis.
 enfant-m|Je suis triste.
-papa|Tu es triste. C'est permis.
-papa|Pleurer est permis.
-narrateur|Victorino pleure un peu.
-narrateur|Les larmes coulent. Elles sont chaudes.
-maman|Je t'écoute, Victorino.
+narrateur|Victorino pleure un peu, sans crier.
+narrateur|Les larmes coulent sur ses joues.
+papa|Tu as les yeux chauds, Victorino ?
+enfant-m|Oui, papa.
+narrateur|Papa s'accroupit à la même hauteur.
+maman|Tes mains sont chaudes, Victorino ?
+enfant-m|Un peu, maman.
 enfant-m|Je veux un câlin.
-papa|Viens. Un câlin.
+maman|Viens.
 narrateur|Papa ouvre les bras.
-narrateur|Victorino se blottit.
-narrateur|Le câlin est chaud.
-narrateur|Le pull de papa sent le savon.
-maman|Tu as dit : je suis triste.
-maman|Bravo. Tu as demandé un câlin.
-papa|Pleurer est permis, Victorino.
-enfant-m|Le câlin aide.
-papa|Oui. Le câlin aide.
-narrateur|Plus tard, au salon.
-narrateur|Le canapé a une couverture rayée.
-narrateur|Une tasse vide attend sur la table.
-narrateur|Amir boutonne son manteau.
-enfant-m|Je rentre chez moi.
-narrateur|Amir part, tout doucement.
-narrateur|Victorino sent encore sa gorge.
-enfant-m|Je suis triste.
-maman|Tu es triste. C'est permis.
-maman|Pleurer est permis.
-enfant-m|Je veux un câlin.
-maman|Viens. Un câlin.
-narrateur|Maman le serre.
-narrateur|Ses épaules se desserrent.
-papa|Bravo. Tu as dit tes larmes.
-papa|On peut demander un câlin.
-enfant-m|Le train, puis Amir.
-maman|Le train, c'était pareil.
-narrateur|La poussière danse encore.</t>
+narrateur|Victorino se blottit contre papa.
+narrateur|Le câlin est chaud, près du cou.
+narrateur|Ça sent le savon de papa.
+narrateur|L'éclat de coffre tremble, puis tient.</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>coffre</t>
         </is>
       </c>
     </row>
@@ -1410,12 +1432,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Victorino a les yeux chauds. Que dit-il ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;&lt;emphasis level="moderate"&gt;Victorino&lt;/emphasis&gt; a les yeux chauds. Que dit-il ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Étienne a les yeux chauds. Que dit-il ?</t>
+          <t>&lt;soft&gt;&lt;slow&gt;&lt;emphasis&gt;Victorino&lt;/emphasis&gt; a les yeux chauds. Que dit-il ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1440,7 +1462,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Étienne peut demander un câlin. Que dit-il ?</t>
+          <t>Victorino peut demander un câlin. Que dit-il ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1478,18 +1500,18 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.24</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1504,34 +1526,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>Victorino</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1540,28 +1566,29 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=victorino_a_les_yeux_chauds_que_dit_il; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Victorino a les yeux chauds. Que dit-il ?</t>
+          <t>narrateur|Victorino a les yeux chauds.
+narrateur|Que dit-il ?</t>
         </is>
       </c>
     </row>
@@ -1588,17 +1615,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Victorino sèche une larme avec sa manche. Je suis triste. Oui. Et pleurer est permis. Un câlin de papa ou maman aide. Bravo. Tu as dit ce que tu sentais. Tu veux encore un câlin ? Encore un peu. Maman le serre, sans se presser. La couverture rayée est douce.</t>
+          <t>Victorino reste contre papa, un moment. Le train, maintenant. Les mots se bousculent dans sa bouche. Je le prends. Victorino avance les mains, trop vite. Puis il s'arrête. Victorino refuse de foncer. Il referme la bouche. Personne ne parle. Il observe la chambre, un instant. Il écoute le coffre, près du tapis. Tu restes un peu, Victorino ? Oui, papa. Merci, Victorino. Papa reste à la même hauteur. Le câlin est tiède, sous les bras. Il est chaud. On va au salon ? Oui, Amir. La poitrine de Victorino ralentit un peu. Tes joues sont mouillées, Victorino ? Un peu, maman. On cherche sans se presser ? Oui. Maman essuie une larme du pouce. Ça pique les yeux. Le ventre de Victorino se desserre. On porte le coffre au salon ? Oui, papa. Je prends un bord. Papa soulève le coffre, sans se bousculer. Le train, papa. On y va, sans se presser. Vous marchez jusqu'au salon ? Oui, maman.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Victorino sèche une larme avec sa manche. Je suis triste. Oui. Et pleurer est permis. Un câlin de papa ou maman aide. Bravo. Tu as dit ce que tu sentais. Tu veux encore un câlin ? Encore un peu. Maman le serre, sans se presser. La couverture rayée est douce.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Victorino reste contre papa, un moment. Le train, maintenant. Les mots se bousculent dans sa bouche. Je le prends. Victorino avance les mains, trop vite. Puis il s'arrête. Victorino refuse de foncer. Il referme la bouche. Personne ne parle. Il observe la chambre, un instant. Il écoute le coffre, près du tapis. Tu restes un peu, Victorino ? Oui, papa. Merci, Victorino. Papa reste à la même hauteur. Le &lt;emphasis level="moderate"&gt;câlin&lt;/emphasis&gt; est tiède, sous les bras. Il est chaud. On va au salon ? Oui, Amir. La poitrine de Victorino ralentit un peu. Tes joues sont mouillées, Victorino ? Un peu, maman. On cherche sans se presser ? Oui. Maman essuie une larme du pouce. Ça pique les yeux. Le ventre de Victorino se desserre. On porte le coffre au salon ? Oui, papa. Je prends un bord. Papa soulève le coffre, sans se bousculer. Le train, papa. On y va, sans se presser. Vous marchez jusqu'au salon ? Oui, maman.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Étienne a nommé : &lt;emphasis&gt;triste&lt;/emphasis&gt;. Pleurer est permis. Un câlin de papa ou maman aide. [pause]</t>
+          <t>Victorino reste contre papa, un moment. Le train, maintenant. Les mots se bousculent dans sa bouche. Je le prends. Victorino avance les mains, trop vite. Puis il s'arrête. Victorino refuse de foncer. Il referme la bouche. Personne ne parle. Il observe la chambre, un instant. Il écoute le coffre, près du tapis. Tu restes un peu, Victorino ? Oui, papa. Merci, Victorino. Papa reste à la même hauteur. Le &lt;emphasis&gt;câlin&lt;/emphasis&gt; est tiède, sous les bras. Il est chaud. On va au salon ? Oui, Amir. La poitrine de Victorino ralentit un peu. Tes joues sont mouillées, Victorino ? Un peu, maman. On cherche sans se presser ? Oui. Maman essuie une larme du pouce. Ça pique les yeux. Le ventre de Victorino se desserre. On porte le coffre au salon ? Oui, papa. Je prends un bord. Papa soulève le coffre, sans se bousculer. Le train, papa. On y va, sans se presser. Vous marchez jusqu'au salon ? Oui, maman. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1645,7 +1672,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1653,10 +1680,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.12</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1679,30 +1706,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>triste</t>
+          <t>câlin</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1711,10 +1738,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1727,20 +1754,46 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis soulagement; intensite=2; destinataire=enfant; sous_texte=il_demande_un_calin_sans_slogan; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Victorino sèche une larme avec sa manche.
-enfant-m|Je suis triste.
-papa|Oui. Et pleurer est permis.
-maman|Un câlin de papa ou maman aide.
-papa|Bravo. Tu as dit ce que tu sentais.
-papa|Tu veux encore un câlin ?
-enfant-m|Encore un peu.
-narrateur|Maman le serre, sans se presser.
-narrateur|La couverture rayée est douce.</t>
+          <t>narrateur|Victorino reste contre papa, un moment.
+enfant-m|Le train, maintenant.
+narrateur|Les mots se bousculent dans sa bouche.
+enfant-m|Je le prends.
+narrateur|Victorino avance les mains, trop vite.
+narrateur|Puis il s'arrête.
+narrateur|Victorino refuse de foncer.
+narrateur|Il referme la bouche.
+narrateur|Personne ne parle.
+narrateur|Il observe la chambre, un instant.
+narrateur|Il écoute le coffre, près du tapis.
+papa|Tu restes un peu, Victorino ?
+enfant-m|Oui, papa.
+papa|Merci, Victorino.
+narrateur|Papa reste à la même hauteur.
+maman|Le câlin est tiède, sous les bras.
+enfant-m|Il est chaud.
+copain|On va au salon ?
+enfant-m|Oui, Amir.
+narrateur|La poitrine de Victorino ralentit un peu.
+maman|Tes joues sont mouillées, Victorino ?
+enfant-m|Un peu, maman.
+papa|On cherche sans se presser ?
+enfant-m|Oui.
+narrateur|Maman essuie une larme du pouce.
+enfant-m|Ça pique les yeux.
+narrateur|Le ventre de Victorino se desserre.
+papa|On porte le coffre au salon ?
+enfant-m|Oui, papa.
+copain|Je prends un bord.
+narrateur|Papa soulève le coffre, sans se bousculer.
+enfant-m|Le train, papa.
+papa|On y va, sans se presser.
+maman|Vous marchez jusqu'au salon ?
+enfant-m|Oui, maman.</t>
         </is>
       </c>
     </row>
@@ -1767,17 +1820,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Papa se baisse près du canapé. Le train. Il était dessous. Mon train ! Victorino le pose près de lui. Le bois est lisse et tiède. Tu as bien demandé le câlin. Je suis moins triste. Le câlin est encore là. Ils restent près du canapé, tout calmes.</t>
+          <t>Ils posent le coffre près du canapé. Une tasse vide attend sur la table. Le train, maintenant ! Amir boutonne son manteau, trop vite. Je rentre chez moi. Pas maintenant ! Le train n'est pas là, au salon. Victorino avance trop vite vers la porte. Amir, attends ! Puis il s'arrête net. Victorino refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe le coffre, un instant. Il écoute le salon, près du canapé. Sur le couvercle, un éclat de coffre luit. Là, sur le bois. On tient le bord ? Oui, papa. Papa ouvre le coffre, sans se presser. Un rail glisse, puis un wagon. Le train ! Le train en bois reste coincé sous un rabat. Il est coincé ! Tu le vois, le bois ? Oui, maman. Victorino veut tirer, tout de suite. Puis il lâche le rabat. J'y vais, Victorino ? Oui, papa. Papa glisse la main, sans se presser. Le train faillit rester coincé. Doucement. Je le tiens. Papa tire le train, tout petit à petit. Mon train ! Victorino le serre contre lui. Le bois est tiède, Victorino ? Un peu. Une roue est un peu marquée. Elle a une trace. Tu vois le point, Victorino ? Oui, papa. On reste près du coffre ? Oui.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Papa se baisse près du canapé. Le train. Il était dessous. Mon train ! Victorino le pose près de lui. Le bois est lisse et tiède. Tu as bien demandé le câlin. Je suis moins triste. Le câlin est encore là. Ils restent près du canapé, tout calmes.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Ils posent le coffre près du canapé. Une tasse vide attend sur la table. Le train, maintenant ! Amir boutonne son manteau, trop vite. Je rentre chez moi. Pas maintenant ! Le train n'est pas là, au salon. Victorino avance trop vite vers la porte. Amir, attends ! Puis il s'arrête net. Victorino refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe le coffre, un instant. Il écoute le salon, près du canapé. Sur le couvercle, un &lt;emphasis level="moderate"&gt;éclat de coffre&lt;/emphasis&gt; luit. Là, sur le bois. On tient le bord ? Oui, papa. Papa ouvre le coffre, sans se presser. Un rail glisse, puis un wagon. Le train ! Le train en bois reste coincé sous un rabat. Il est coincé ! Tu le vois, le bois ? Oui, maman. Victorino veut tirer, tout de suite. Puis il lâche le rabat. J'y vais, Victorino ? Oui, papa. Papa glisse la main, sans se presser. Le train faillit rester coincé. Doucement. Je le tiens. Papa tire le train, tout petit à petit. Mon train ! Victorino le serre contre lui. Le bois est tiède, Victorino ? Un peu. Une roue est un peu marquée. Elle a une trace. Tu vois le point, Victorino ? Oui, papa. On reste près du coffre ? Oui.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Papa retrouve le train sous le canapé. Étienne le pose près de lui. [pause]</t>
+          <t>Ils posent le coffre près du canapé. Une tasse vide attend sur la table. Le train, maintenant ! Amir boutonne son manteau, trop vite. Je rentre chez moi. Pas maintenant ! Le train n'est pas là, au salon. Victorino avance trop vite vers la porte. Amir, attends ! Puis il s'arrête net. Victorino refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe le coffre, un instant. Il écoute le salon, près du canapé. Sur le couvercle, un &lt;emphasis&gt;éclat de coffre&lt;/emphasis&gt; luit. Là, sur le bois. On tient le bord ? Oui, papa. Papa ouvre le coffre, sans se presser. Un rail glisse, puis un wagon. Le train ! Le train en bois reste coincé sous un rabat. Il est coincé ! Tu le vois, le bois ? Oui, maman. Victorino veut tirer, tout de suite. Puis il lâche le rabat. J'y vais, Victorino ? Oui, papa. Papa glisse la main, sans se presser. Le train faillit rester coincé. Doucement. Je le tiens. Papa tire le train, tout petit à petit. Mon train ! Victorino le serre contre lui. Le bois est tiède, Victorino ? Un peu. Une roue est un peu marquée. Elle a une trace. Tu vois le point, Victorino ? Oui, papa. On reste près du coffre ? Oui. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1824,7 +1877,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1832,10 +1885,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.12</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1856,28 +1909,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de coffre</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1886,10 +1943,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1900,18 +1957,58 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=amir_rentre_train_perdu_il_refuse_de_foncer; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Papa se baisse près du canapé.
-papa|Le train. Il était dessous.
+          <t>narrateur|Ils posent le coffre près du canapé.
+narrateur|Une tasse vide attend sur la table.
+enfant-m|Le train, maintenant !
+narrateur|Amir boutonne son manteau, trop vite.
+copain|Je rentre chez moi.
+enfant-m|Pas maintenant !
+narrateur|Le train n'est pas là, au salon.
+narrateur|Victorino avance trop vite vers la porte.
+enfant-m|Amir, attends !
+narrateur|Puis il s'arrête net.
+narrateur|Victorino refuse de foncer, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Personne ne dit la suite.
+narrateur|Il observe le coffre, un instant.
+narrateur|Il écoute le salon, près du canapé.
+narrateur|Sur le couvercle, un éclat de coffre luit.
+enfant-m|Là, sur le bois.
+papa|On tient le bord ?
+enfant-m|Oui, papa.
+narrateur|Papa ouvre le coffre, sans se presser.
+narrateur|Un rail glisse, puis un wagon.
+enfant-m|Le train !
+narrateur|Le train en bois reste coincé sous un rabat.
+enfant-m|Il est coincé !
+maman|Tu le vois, le bois ?
+enfant-m|Oui, maman.
+narrateur|Victorino veut tirer, tout de suite.
+narrateur|Puis il lâche le rabat.
+papa|J'y vais, Victorino ?
+enfant-m|Oui, papa.
+narrateur|Papa glisse la main, sans se presser.
+narrateur|Le train faillit rester coincé.
+enfant-m|Doucement.
+papa|Je le tiens.
+narrateur|Papa tire le train, tout petit à petit.
 enfant-m|Mon train !
-narrateur|Victorino le pose près de lui.
-narrateur|Le bois est lisse et tiède.
-maman|Tu as bien demandé le câlin.
-enfant-m|Je suis moins triste.
-papa|Le câlin est encore là.
-narrateur|Ils restent près du canapé, tout calmes.</t>
+narrateur|Victorino le serre contre lui.
+maman|Le bois est tiède, Victorino ?
+enfant-m|Un peu.
+papa|Une roue est un peu marquée.
+enfant-m|Elle a une trace.
+papa|Tu vois le point, Victorino ?
+enfant-m|Oui, papa.
+papa|On reste près du coffre ?
+enfant-m|Oui.</t>
         </is>
       </c>
     </row>
@@ -1938,17 +2035,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>J'ai dit : je suis triste. J'ai eu un câlin. Pleurer est permis. Bravo, Victorino.</t>
+          <t>Ils restent près du coffre. Maman essuie un peu de vernis. Amir est rentré, papa. Tu l'as vu, toi ? Oui, près de la porte. On est bien, ici. Victorino tapote le bois du doigt. Il a une roue marquée. Tu la vois, la trace ? Oui, maman. Le train est resté, Victorino. Oui, avec la roue. Ça sent le vernis, un peu tiède. Et le bois, maman. Oui, dans l'air. Le salon est doux, Victorino ? Oui, papa. Le train reste contre le coffre. Un éclat de coffre tient sur le bois.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>J'ai dit : je suis triste. J'ai eu un câlin. Pleurer est permis. Bravo, Victorino.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près du coffre. Maman essuie un peu de vernis. Amir est rentré, papa. Tu l'as vu, toi ? Oui, près de la porte. On est bien, ici. Victorino tapote le bois du doigt. Il a une roue marquée. Tu la vois, la trace ? Oui, maman. Le train est resté, Victorino. Oui, avec la roue. Ça sent le vernis, un peu tiède. Et le bois, maman. Oui, dans l'air. Le salon est doux, Victorino ? Oui, papa. Le train reste contre le coffre. Un &lt;emphasis level="moderate"&gt;éclat de coffre&lt;/emphasis&gt; tient sur le bois.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;L'histoire est finie.&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près du coffre. Maman essuie un peu de vernis. Amir est rentré, papa. Tu l'as vu, toi ? Oui, près de la porte. On est bien, ici. Victorino tapote le bois du doigt. Il a une roue marquée. Tu la vois, la trace ? Oui, maman. Le train est resté, Victorino. Oui, avec la roue. Ça sent le vernis, un peu tiède. Et le bois, maman. Oui, dans l'air. Le salon est doux, Victorino ? Oui, papa. Le train reste contre le coffre. Un &lt;emphasis&gt;éclat de coffre&lt;/emphasis&gt; tient sur le bois.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -1995,18 +2092,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.2</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2015,12 +2112,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2029,17 +2126,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de coffre</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2048,11 +2149,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2061,27 +2162,46 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_soulagement; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_bois; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-m|J'ai dit : je suis triste.
-enfant-m|J'ai eu un câlin.
-maman|Pleurer est permis.
-papa|Bravo, Victorino.</t>
+          <t>narrateur|Ils restent près du coffre.
+narrateur|Maman essuie un peu de vernis.
+enfant-m|Amir est rentré, papa.
+papa|Tu l'as vu, toi ?
+enfant-m|Oui, près de la porte.
+maman|On est bien, ici.
+narrateur|Victorino tapote le bois du doigt.
+enfant-m|Il a une roue marquée.
+maman|Tu la vois, la trace ?
+enfant-m|Oui, maman.
+papa|Le train est resté, Victorino.
+enfant-m|Oui, avec la roue.
+narrateur|Ça sent le vernis, un peu tiède.
+enfant-m|Et le bois, maman.
+maman|Oui, dans l'air.
+papa|Le salon est doux, Victorino ?
+enfant-m|Oui, papa.
+narrateur|Le train reste contre le coffre.
+narrateur|Un éclat de coffre tient sur le bois.</t>
         </is>
       </c>
     </row>
@@ -2102,7 +2222,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2152,6 +2272,13 @@
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>